<commit_message>
Add STS test cases for tags, nodeHandle, propertyHandle, propertyTerms PSDC
</commit_message>
<xml_diff>
--- a/InputFiles/API/MDB/CypherQueries.xlsx
+++ b/InputFiles/API/MDB/CypherQueries.xlsx
@@ -1,169 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leungvw/git2/Commons_Automation/InputFiles/API/MDB/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40C3FF49-3D02-F642-8397-7FA1B2FC4524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="12500" yWindow="-23600" windowWidth="39620" windowHeight="17800" xr2:uid="{E31DFAE0-8367-D64E-B72E-FBCDBE56359A}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12500" yWindow="-23600" windowWidth="39620" windowHeight="17800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="queries" sheetId="2" r:id="rId1"/>
+    <sheet name="queries" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>key</t>
-  </si>
-  <si>
-    <t>cypher</t>
-  </si>
-  <si>
-    <t>verifyModelNodes</t>
-  </si>
-  <si>
-    <t>verifyModels</t>
-  </si>
-  <si>
-    <t>verifyModelVersions</t>
-  </si>
-  <si>
-    <t>verifyModelNodeProperties</t>
-  </si>
-  <si>
-    <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
-MATCH (n)-[:has_property]-&gt;(p:property)
-RETURN DISTINCT
-  p.model        AS model,
-  p.version      AS version,
-  n.handle       AS node,
-  p.handle       AS handle,
-  p.nanoid       AS nanoid,
-  p.is_key       AS is_key,
-  p.is_strict    AS is_strict,
-  p.is_nullable  AS is_nullable,
-  p.is_required  AS is_required,
-  p.value_domain AS value_domain,
-  p.desc         AS desc
-ORDER BY handle</t>
-  </si>
-  <si>
-    <t>MATCH (n:node { model: $handle }) 
-RETURN DISTINCT 
-n.version AS version 
-ORDER BY version</t>
-  </si>
-  <si>
-    <t>MATCH (n:node { model: $handle, version: $version }) 
-RETURN n.model  AS model, 
-n.handle  AS handle, 
-n.version AS version, 
-n.nanoid  AS nanoid 
-ORDER BY model, handle, version, nanoid</t>
-  </si>
-  <si>
-    <t>MATCH (m:model) 
-RETURN m.handle AS handle, 
-m.version AS version, 
-m.nanoid AS nanoid, 
-m.is_latest_version AS is_latest_version 
-ORDER BY handle, version</t>
-  </si>
-  <si>
-    <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
-			MATCH (n)-[:has_property]-&gt;(p:property)
-			RETURN p</t>
-  </si>
-  <si>
-    <t>verifyModelNodePropertiesEmpty</t>
-  </si>
-  <si>
-    <t>verifyModelNodePropertyTerms</t>
-  </si>
-  <si>
-    <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
-MATCH (n)-[:has_property]-&gt;(p:property { handle: $propHandle })
-MATCH (p)-[:has_value_set]-&gt;(vs:value_set)
-MATCH (vs)-[:has_term]-&gt;(t:term)
-RETURN
-  n.model          AS model,
-  n.version        AS version,
-  n.handle         AS node,
-  p.handle         AS property,
-  t.value          AS value,
-  t.handle         AS handle,
-  t.origin_name    AS origin_name,
-  t.origin_version AS origin_version,
-  t.origin_id      AS origin_id,
-  t.nanoid         AS nanoid
-ORDER BY value, nanoid</t>
-  </si>
-  <si>
-    <t>verifyModelNodePropertyTermsEmpty</t>
-  </si>
-  <si>
-    <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
-MATCH (n)-[:has_property]-&gt;(p:property { handle: $propHandle })
-MATCH (p)-[:has_value_set]-&gt;(vs:value_set)
-MATCH (vs)-[:has_term]-&gt;(t:term)
-RETURN t.nanoid AS nanoid
-LIMIT 1</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -182,29 +59,88 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -524,76 +460,219 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D8CE0E7-003B-DB4B-B327-82B56A12C61B}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="43.83203125" customWidth="1"/>
-    <col min="2" max="2" width="166" customWidth="1"/>
+    <col width="43.83203125" customWidth="1" min="1" max="1"/>
+    <col width="166" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="102" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="102" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="68" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="255" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="51" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="272" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="102" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>15</v>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>cypher</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="102" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>verifyModels</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>MATCH (m:model) 
+RETURN m.handle AS handle, 
+m.version AS version, 
+m.nanoid AS nanoid, 
+m.is_latest_version AS is_latest_version 
+ORDER BY handle, version</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="102" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>verifyModelNodes</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>MATCH (n:node { model: $handle, version: $version }) 
+RETURN n.model  AS model, 
+n.handle  AS handle, 
+n.version AS version, 
+n.nanoid  AS nanoid 
+ORDER BY model, handle, version, nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="68" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>verifyModelVersions</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>MATCH (n:node { model: $handle }) 
+RETURN DISTINCT 
+n.version AS version 
+ORDER BY version</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="255" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>verifyModelNodeProperties</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
+MATCH (n)-[:has_property]-&gt;(p:property)
+RETURN DISTINCT
+  p.model        AS model,
+  p.version      AS version,
+  n.handle       AS node,
+  p.handle       AS handle,
+  p.nanoid       AS nanoid,
+  p.is_key       AS is_key,
+  p.is_strict    AS is_strict,
+  p.is_nullable  AS is_nullable,
+  p.is_required  AS is_required,
+  p.value_domain AS value_domain,
+  p.desc         AS desc
+ORDER BY handle</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="51" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>verifyModelNodePropertiesEmpty</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
+			MATCH (n)-[:has_property]-&gt;(p:property)
+			RETURN p</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="272" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>verifyModelNodePropertyTerms</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
+MATCH (n)-[:has_property]-&gt;(p:property { handle: $propHandle })
+MATCH (p)-[:has_value_set]-&gt;(vs:value_set)
+MATCH (vs)-[:has_term]-&gt;(t:term)
+RETURN
+  n.model          AS model,
+  n.version        AS version,
+  n.handle         AS node,
+  p.handle         AS property,
+  t.value          AS value,
+  t.handle         AS handle,
+  t.origin_name    AS origin_name,
+  t.origin_version AS origin_version,
+  t.origin_id      AS origin_id,
+  t.nanoid         AS nanoid
+ORDER BY value, nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="102" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>verifyModelNodePropertyTermsEmpty</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
+MATCH (n)-[:has_property]-&gt;(p:property { handle: $propHandle })
+MATCH (p)-[:has_value_set]-&gt;(vs:value_set)
+MATCH (vs)-[:has_term]-&gt;(t:term)
+RETURN t.nanoid AS nanoid
+LIMIT 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>verifyTags</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MATCH (t:tag)
+RETURN t.key AS key,
+       t.value AS value,
+       t.nanoid AS nanoid
+ORDER BY key, value, nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>verifyModelNode</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
+RETURN n.model  AS model,
+       n.handle  AS handle,
+       n.version AS version,
+       n.nanoid  AS nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>verifyModelNodeProperty</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MATCH (n:node { model: $modelHandle, version: $versionString, handle: $nodeHandle })
+MATCH (n)-[:has_property]-&gt;(p:property { handle: $propHandle })
+RETURN DISTINCT
+  p.model        AS model,
+  p.version      AS version,
+  n.handle       AS node,
+  p.handle       AS handle,
+  p.nanoid       AS nanoid,
+  p.is_key       AS is_key,
+  p.is_strict    AS is_strict,
+  p.is_nullable  AS is_nullable,
+  p.is_required  AS is_required,
+  p.value_domain AS value_domain,
+  p.desc         AS desc
+ORDER BY handle</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MDB - add remaining tag tests
</commit_message>
<xml_diff>
--- a/InputFiles/API/MDB/CypherQueries.xlsx
+++ b/InputFiles/API/MDB/CypherQueries.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="43.83203125" customWidth="1" min="1" max="1"/>
@@ -675,6 +675,131 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>verifyTagValues</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MATCH (t:tag)
+WHERE t.key = $key
+RETURN DISTINCT t.value AS value
+ORDER BY value</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>verifyTagKeyValueEntities</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MATCH (t:tag)
+WHERE t.key = $key AND (t.value = $value OR (t.value IS NOT NULL AND toString(t.value) = $value))
+MATCH (p:property)-[:has_tag]-&gt;(t)
+RETURN DISTINCT
+  p.model        AS model,
+  p.version      AS version,
+  p.handle       AS handle,
+  p.nanoid       AS nanoid,
+  p.is_key       AS is_key,
+  p.is_strict    AS is_strict,
+  p.is_nullable  AS is_nullable,
+  p.is_required  AS is_required,
+  p.value_domain AS value_domain,
+  p.item_domain  AS item_domain,
+  p.units        AS units,
+  p.pattern      AS pattern,
+  p.desc         AS desc
+ORDER BY model, version, handle, nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>verifyTagKeyValueEntitiesNode</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MATCH (t:tag)
+WHERE t.key = $key AND (t.value = $value OR (t.value IS NOT NULL AND toString(t.value) = $value))
+MATCH (n:node)-[:has_tag]-&gt;(t)
+RETURN DISTINCT
+  n.model  AS model,
+  n.handle AS handle,
+  n.version AS version,
+  n.nanoid AS nanoid
+ORDER BY model, handle, version, nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>verifyTagKeyValueEntitiesTerm</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MATCH (t:tag)
+WHERE t.key = $key AND (t.value = $value OR (t.value IS NOT NULL AND toString(t.value) = $value))
+MATCH (tm:term)-[:has_tag]-&gt;(t)
+RETURN DISTINCT
+  tm.value AS value,
+  tm.origin_name AS origin_name,
+  tm.handle AS handle,
+  tm.origin_version AS origin_version,
+  tm.origin_id AS origin_id,
+  tm.nanoid AS nanoid
+ORDER BY value, nanoid, handle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>verifyTagKeyValueEntitiesConcept</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MATCH (t:tag)
+WHERE t.key = $key AND (t.value = $value OR (t.value IS NOT NULL AND toString(t.value) = $value))
+MATCH (c:concept)-[:has_tag]-&gt;(t)
+RETURN DISTINCT
+  c.handle AS handle,
+  c.version AS version,
+  c.nanoid AS nanoid
+ORDER BY handle, version, nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>verifyTagKeyValueEntitiesRelationship</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MATCH (t:tag)
+WHERE t.key = $key AND (t.value = $value OR (t.value IS NOT NULL AND toString(t.value) = $value))
+MATCH (rel:relationship)-[:has_tag]-&gt;(t)
+RETURN DISTINCT
+  rel.model AS model,
+  rel.handle AS handle,
+  rel.version AS version,
+  rel.nanoid AS nanoid
+ORDER BY model, handle, version, nanoid</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add parity tests for EDP endpoints
</commit_message>
<xml_diff>
--- a/InputFiles/API/MDB/CypherQueries.xlsx
+++ b/InputFiles/API/MDB/CypherQueries.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="43.83203125" customWidth="1" min="1" max="1"/>
@@ -800,6 +800,63 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>verifyEdpsByOrigin</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MATCH (t:term {origin_name: $origin_name})-[:specifies_value_set]-&gt;(:value_set)
+RETURN DISTINCT
+  t.value AS value,
+  t.origin_name AS origin_name,
+  t.handle AS handle,
+  t.origin_version AS origin_version,
+  t.origin_id AS origin_id,
+  t.nanoid AS nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>verifyEdpTerms</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MATCH (:term {origin_name: $origin_name, origin_id: $origin_id, origin_version: $origin_version})
+      -[:specifies_value_set]-&gt;(:value_set)-[:has_term]-&gt;(t:term)
+RETURN t.value AS value,
+       t.origin_name AS origin_name,
+       t.handle AS handle,
+       t.origin_version AS origin_version,
+       t.origin_id AS origin_id,
+       t.nanoid AS nanoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>verifyEdpTermsEmpty</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MATCH (:term {origin_name: $origin_name, origin_id: $origin_id, origin_version: $origin_version})
+      -[:specifies_value_set]-&gt;(:value_set)-[:has_term]-&gt;(t:term)
+RETURN t.value AS value,
+       t.origin_name AS origin_name,
+       t.handle AS handle,
+       t.origin_version AS origin_version,
+       t.origin_id AS origin_id,
+       t.nanoid AS nanoid</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add parity test for newly added edps properties endpoint
</commit_message>
<xml_diff>
--- a/InputFiles/API/MDB/CypherQueries.xlsx
+++ b/InputFiles/API/MDB/CypherQueries.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="43.83203125" customWidth="1" min="1" max="1"/>
@@ -857,6 +857,68 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>verifyEdpProperties</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MATCH (p:property)-[:has_value_set]-&gt;(:value_set)
+      &lt;-[:specifies_value_set]-(:term {
+        origin_name: $origin_name,
+        origin_id: $origin_id,
+        origin_version: $origin_version
+      })
+RETURN DISTINCT
+  p.model AS model,
+  p.version AS version,
+  p.handle AS handle,
+  p.nanoid AS nanoid,
+  p.is_key AS is_key,
+  p.is_strict AS is_strict,
+  p.is_nullable AS is_nullable,
+  p.is_required AS is_required,
+  p.value_domain AS value_domain,
+  p.item_domain AS item_domain,
+  p.units AS units,
+  p.pattern AS pattern,
+  p.desc AS desc</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>verifyEdpPropertiesEmpty</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MATCH (p:property)-[:has_value_set]-&gt;(:value_set)
+      &lt;-[:specifies_value_set]-(:term {
+        origin_name: $origin_name,
+        origin_id: $origin_id,
+        origin_version: $origin_version
+      })
+RETURN DISTINCT
+  p.model AS model,
+  p.version AS version,
+  p.handle AS handle,
+  p.nanoid AS nanoid,
+  p.is_key AS is_key,
+  p.is_strict AS is_strict,
+  p.is_nullable AS is_nullable,
+  p.is_required AS is_required,
+  p.value_domain AS value_domain,
+  p.item_domain AS item_domain,
+  p.units AS units,
+  p.pattern AS pattern,
+  p.desc AS desc</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>